<commit_message>
New Notebooks, new startified group cross validation, added regression for Prezado only
</commit_message>
<xml_diff>
--- a/data/raw/electrons-protons/PREZADO-MICE-FLASH-INVIVO-NORMAL.xlsx
+++ b/data/raw/electrons-protons/PREZADO-MICE-FLASH-INVIVO-NORMAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\silvi\Desktop\Tesi\Dataset\Elec-Prot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\silvi\Desktop\mastersthesis\data\raw\electrons-protons\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E812FDA-ADBF-4AD3-8F7F-2EC161113B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FDA360-53B6-43E1-BD1D-1EEFB6567CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="51">
   <si>
     <t>Title</t>
   </si>
@@ -186,9 +186,6 @@
   </si>
   <si>
     <t>Rat brain</t>
-  </si>
-  <si>
-    <t>Oxygen supplementation can block FLASH effect</t>
   </si>
   <si>
     <t>Anesthetic Oxygen Use and Sex Are Critical Factors</t>
@@ -3295,7 +3292,7 @@
     </row>
     <row r="53" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B53" s="2">
         <v>257</v>
@@ -3348,7 +3345,7 @@
     </row>
     <row r="54" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B54" s="2">
         <v>200</v>
@@ -3401,7 +3398,7 @@
     </row>
     <row r="55" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B55" s="2">
         <v>200</v>

</xml_diff>